<commit_message>
chore: remove unused ReportPeriod import and align 2020 label with DuckDB
</commit_message>
<xml_diff>
--- a/data/000423_label/东阿阿胶_000423_2020.xlsx
+++ b/data/000423_label/东阿阿胶_000423_2020.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="合并资产负债表" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="合并利润表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="合并现金流量表" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并资产负债表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并利润表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并现金流量表" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2460,10 +2460,8 @@
           <t>（二）将重分类进损益的其他综合收益</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>60,519.45</t>
-        </is>
+      <c r="B53" s="3" t="n">
+        <v>60519.45</v>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
@@ -2526,10 +2524,8 @@
           <t>6.外币财务报表折算差额</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>60,519.45</t>
-        </is>
+      <c r="B59" s="3" t="n">
+        <v>60519.45</v>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
@@ -2621,10 +2617,8 @@
           <t>（一）基本每股收益</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>0.07</t>
-        </is>
+      <c r="B66" s="3" t="n">
+        <v>0.07000000000000001</v>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
@@ -2638,10 +2632,8 @@
           <t>（二）稀释每股收益</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>0.07</t>
-        </is>
+      <c r="B67" s="3" t="n">
+        <v>0.07000000000000001</v>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>

</xml_diff>